<commit_message>
Add Cube demo guide, 40 more criteria, weighted score sheet, round-3 build-out and gap tests; add net_revenue and related metrics, per-user identity in MCP wrapper
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan-1/success-criteria-grid.xlsx
+++ b/docs/plan-1/success-criteria-grid.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Success Criteria" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Weighted Score" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -16,8 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="12">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -99,8 +102,26 @@
       <color rgb="FF475569"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -155,8 +176,28 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003B1D3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -256,6 +297,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BBBBBB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BBBBBB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BBBBBB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BBBBBB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -267,7 +322,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -428,6 +483,41 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="14" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1998,4 +2088,714 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" style="27" min="1" max="1"/>
+    <col width="10" customWidth="1" style="27" min="2" max="2"/>
+    <col width="22" customWidth="1" style="27" min="3" max="3"/>
+    <col width="22" customWidth="1" style="27" min="4" max="4"/>
+    <col width="22" customWidth="1" style="27" min="5" max="5"/>
+    <col width="22" customWidth="1" style="27" min="6" max="6"/>
+    <col width="70" customWidth="1" style="27" min="7" max="7"/>
+    <col width="9" customWidth="1" style="27" min="9" max="9"/>
+    <col width="9" customWidth="1" style="27" min="10" max="10"/>
+    <col width="9" customWidth="1" style="27" min="11" max="11"/>
+    <col width="9" customWidth="1" style="27" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="57" t="inlineStr">
+        <is>
+          <t>Weighted score: 4 routes x 8 criteria</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1" s="27">
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>PROPOSED weights, not set by leadership (the success criteria say leadership sets them). Yellow cells are inputs: change weights, scores or the two switches and every result updates. Scores are 0-3 from the scoring matrix (docs/plan-1/scoring-matrix.md); blank = not scored yet, and is never counted as zero in the headline score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="I3" s="69" t="inlineStr">
+        <is>
+          <t>Helper: 1 if the route has a score for the criterion</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1" s="27">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B4" s="59" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="C4" s="59" t="inlineStr">
+        <is>
+          <t>1. Claude on its own</t>
+        </is>
+      </c>
+      <c r="D4" s="59" t="inlineStr">
+        <is>
+          <t>2. Claude + 3rd-party layer (Cube)</t>
+        </is>
+      </c>
+      <c r="E4" s="59" t="inlineStr">
+        <is>
+          <t>3. Claude + Omni</t>
+        </is>
+      </c>
+      <c r="F4" s="59" t="inlineStr">
+        <is>
+          <t>4. Omni (+ Claude)</t>
+        </is>
+      </c>
+      <c r="G4" s="59" t="inlineStr">
+        <is>
+          <t>Where the score comes from</t>
+        </is>
+      </c>
+      <c r="I4" s="70" t="inlineStr">
+        <is>
+          <t>scored 1</t>
+        </is>
+      </c>
+      <c r="J4" s="70" t="inlineStr">
+        <is>
+          <t>scored 2</t>
+        </is>
+      </c>
+      <c r="K4" s="70" t="inlineStr">
+        <is>
+          <t>scored 3</t>
+        </is>
+      </c>
+      <c r="L4" s="70" t="inlineStr">
+        <is>
+          <t>scored 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44" customHeight="1" s="27">
+      <c r="A5" s="60" t="inlineStr">
+        <is>
+          <t>Setup and upkeep</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="62" t="inlineStr">
+        <is>
+          <t>Asserted/Documented; hours not logged. Counts least, per the success criteria</t>
+        </is>
+      </c>
+      <c r="I5" s="71">
+        <f>IF(ISNUMBER(C5),1,0)</f>
+        <v/>
+      </c>
+      <c r="J5" s="71">
+        <f>IF(ISNUMBER(D5),1,0)</f>
+        <v/>
+      </c>
+      <c r="K5" s="71">
+        <f>IF(ISNUMBER(E5),1,0)</f>
+        <v/>
+      </c>
+      <c r="L5" s="71">
+        <f>IF(ISNUMBER(F5),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="44" customHeight="1" s="27">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>Adding a metric</t>
+        </is>
+      </c>
+      <c r="B6" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G6" s="62" t="inlineStr">
+        <is>
+          <t>Business-user seat: Cube needs an engineer (DE seat 2, business-user seat 1, used here); Omni modeler path Tested, UI path Documented</t>
+        </is>
+      </c>
+      <c r="I6" s="71">
+        <f>IF(ISNUMBER(C6),1,0)</f>
+        <v/>
+      </c>
+      <c r="J6" s="71">
+        <f>IF(ISNUMBER(D6),1,0)</f>
+        <v/>
+      </c>
+      <c r="K6" s="71">
+        <f>IF(ISNUMBER(E6),1,0)</f>
+        <v/>
+      </c>
+      <c r="L6" s="71">
+        <f>IF(ISNUMBER(F6),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="44" customHeight="1" s="27">
+      <c r="A7" s="60" t="inlineStr">
+        <is>
+          <t>Total cost</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7" s="61" t="n"/>
+      <c r="D7" s="61" t="n"/>
+      <c r="E7" s="61" t="n"/>
+      <c r="F7" s="61" t="n"/>
+      <c r="G7" s="62" t="inlineStr">
+        <is>
+          <t>Not measured; left blank</t>
+        </is>
+      </c>
+      <c r="I7" s="71">
+        <f>IF(ISNUMBER(C7),1,0)</f>
+        <v/>
+      </c>
+      <c r="J7" s="71">
+        <f>IF(ISNUMBER(D7),1,0)</f>
+        <v/>
+      </c>
+      <c r="K7" s="71">
+        <f>IF(ISNUMBER(E7),1,0)</f>
+        <v/>
+      </c>
+      <c r="L7" s="71">
+        <f>IF(ISNUMBER(F7),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="44" customHeight="1" s="27">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="B8" s="61" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="63">
+        <f>IF($B$16="Pinned",2,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="63">
+        <f>IF($B$17="Yes",E8,"")</f>
+        <v/>
+      </c>
+      <c r="G8" s="62" t="inlineStr">
+        <is>
+          <t>Tested: 60% / 100% / Omni MCP 37% unguided or 93% pinned. Route 4 uses route 3 as a proxy if the switch is Yes</t>
+        </is>
+      </c>
+      <c r="I8" s="71">
+        <f>IF(ISNUMBER(C8),1,0)</f>
+        <v/>
+      </c>
+      <c r="J8" s="71">
+        <f>IF(ISNUMBER(D8),1,0)</f>
+        <v/>
+      </c>
+      <c r="K8" s="71">
+        <f>IF(ISNUMBER(E8),1,0)</f>
+        <v/>
+      </c>
+      <c r="L8" s="71">
+        <f>IF(ISNUMBER(F8),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="44" customHeight="1" s="27">
+      <c r="A9" s="60" t="inlineStr">
+        <is>
+          <t>Consistency</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" s="63">
+        <f>IF($B$17="Yes",E9,"")</f>
+        <v/>
+      </c>
+      <c r="G9" s="62" t="inlineStr">
+        <is>
+          <t>Tested: 100% / 100% / 90%. Route 1 is consistently wrong</t>
+        </is>
+      </c>
+      <c r="I9" s="71">
+        <f>IF(ISNUMBER(C9),1,0)</f>
+        <v/>
+      </c>
+      <c r="J9" s="71">
+        <f>IF(ISNUMBER(D9),1,0)</f>
+        <v/>
+      </c>
+      <c r="K9" s="71">
+        <f>IF(ISNUMBER(E9),1,0)</f>
+        <v/>
+      </c>
+      <c r="L9" s="71">
+        <f>IF(ISNUMBER(F9),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1" s="27">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>Auditability</t>
+        </is>
+      </c>
+      <c r="B10" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="62" t="inlineStr">
+        <is>
+          <t>SQL visible on routes 1-2; Omni shows SQL and definitions (Tested) and history (Documented)</t>
+        </is>
+      </c>
+      <c r="I10" s="71">
+        <f>IF(ISNUMBER(C10),1,0)</f>
+        <v/>
+      </c>
+      <c r="J10" s="71">
+        <f>IF(ISNUMBER(D10),1,0)</f>
+        <v/>
+      </c>
+      <c r="K10" s="71">
+        <f>IF(ISNUMBER(E10),1,0)</f>
+        <v/>
+      </c>
+      <c r="L10" s="71">
+        <f>IF(ISNUMBER(F10),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1" s="27">
+      <c r="A11" s="60" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="n">
+        <v>15</v>
+      </c>
+      <c r="C11" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="61" t="n"/>
+      <c r="F11" s="61" t="n"/>
+      <c r="G11" s="62" t="inlineStr">
+        <is>
+          <t>Tested FAIL on routes 1-2 (as configured); Omni untested (docs: PASS), blocked by impersonation key</t>
+        </is>
+      </c>
+      <c r="I11" s="71">
+        <f>IF(ISNUMBER(C11),1,0)</f>
+        <v/>
+      </c>
+      <c r="J11" s="71">
+        <f>IF(ISNUMBER(D11),1,0)</f>
+        <v/>
+      </c>
+      <c r="K11" s="71">
+        <f>IF(ISNUMBER(E11),1,0)</f>
+        <v/>
+      </c>
+      <c r="L11" s="71">
+        <f>IF(ISNUMBER(F11),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="44" customHeight="1" s="27">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>Ease of use and sharing</t>
+        </is>
+      </c>
+      <c r="B12" s="61" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="61" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="61" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" s="62" t="inlineStr">
+        <is>
+          <t>Mostly Asserted/Documented; no non-technical trial</t>
+        </is>
+      </c>
+      <c r="I12" s="71">
+        <f>IF(ISNUMBER(C12),1,0)</f>
+        <v/>
+      </c>
+      <c r="J12" s="71">
+        <f>IF(ISNUMBER(D12),1,0)</f>
+        <v/>
+      </c>
+      <c r="K12" s="71">
+        <f>IF(ISNUMBER(E12),1,0)</f>
+        <v/>
+      </c>
+      <c r="L12" s="71">
+        <f>IF(ISNUMBER(F12),1,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>Sum of weights</t>
+        </is>
+      </c>
+      <c r="B13" s="26">
+        <f>SUM(B5:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="26">
+        <f>IF(B13=100,"OK: weights sum to 100","Weights do not sum to 100")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>Switches</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>Omni MCP topic</t>
+        </is>
+      </c>
+      <c r="B16" s="65" t="inlineStr">
+        <is>
+          <t>Unguided</t>
+        </is>
+      </c>
+      <c r="C16" s="26" t="inlineStr">
+        <is>
+          <t>Unguided = the agent picks the topic (36.7% accuracy); Pinned = pointed at the Sales topic (93.3%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr">
+        <is>
+          <t>Use Omni MCP results as proxy for Omni (route 4)</t>
+        </is>
+      </c>
+      <c r="B17" s="65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="inlineStr">
+        <is>
+          <t>Omni's in-app chat was not driven; docs say it shares the MCP's AI pipeline but is not guaranteed identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="64" t="inlineStr">
+        <is>
+          <t>Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="66" t="inlineStr">
+        <is>
+          <t>HEADLINE: weighted score, scored criteria only (% of max)</t>
+        </is>
+      </c>
+      <c r="C20" s="67">
+        <f>SUMPRODUCT($B$5:$B$12,C5:C12)/(3*SUMPRODUCT($B$5:$B$12,I5:I12))</f>
+        <v/>
+      </c>
+      <c r="D20" s="67">
+        <f>SUMPRODUCT($B$5:$B$12,D5:D12)/(3*SUMPRODUCT($B$5:$B$12,J5:J12))</f>
+        <v/>
+      </c>
+      <c r="E20" s="67">
+        <f>SUMPRODUCT($B$5:$B$12,E5:E12)/(3*SUMPRODUCT($B$5:$B$12,K5:K12))</f>
+        <v/>
+      </c>
+      <c r="F20" s="67">
+        <f>SUMPRODUCT($B$5:$B$12,F5:F12)/(3*SUMPRODUCT($B$5:$B$12,L5:L12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="60" t="inlineStr">
+        <is>
+          <t>Coverage: share of total weight that has a score</t>
+        </is>
+      </c>
+      <c r="C21" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,I5:I12)/SUM($B$5:$B$12)</f>
+        <v/>
+      </c>
+      <c r="D21" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,J5:J12)/SUM($B$5:$B$12)</f>
+        <v/>
+      </c>
+      <c r="E21" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,K5:K12)/SUM($B$5:$B$12)</f>
+        <v/>
+      </c>
+      <c r="F21" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,L5:L12)/SUM($B$5:$B$12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>Floor: unscored criteria count as 0</t>
+        </is>
+      </c>
+      <c r="C22" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,C5:C12)/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="D22" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,D5:D12)/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="E22" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,E5:E12)/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="F22" s="68">
+        <f>SUMPRODUCT($B$5:$B$12,F5:F12)/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="60" t="inlineStr">
+        <is>
+          <t>Ceiling: unscored criteria count as 3</t>
+        </is>
+      </c>
+      <c r="C23" s="68">
+        <f>(SUMPRODUCT($B$5:$B$12,C5:C12)+3*(SUM($B$5:$B$12)-SUMPRODUCT($B$5:$B$12,I5:I12)))/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="D23" s="68">
+        <f>(SUMPRODUCT($B$5:$B$12,D5:D12)+3*(SUM($B$5:$B$12)-SUMPRODUCT($B$5:$B$12,J5:J12)))/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="E23" s="68">
+        <f>(SUMPRODUCT($B$5:$B$12,E5:E12)+3*(SUM($B$5:$B$12)-SUMPRODUCT($B$5:$B$12,K5:K12)))/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+      <c r="F23" s="68">
+        <f>(SUMPRODUCT($B$5:$B$12,F5:F12)+3*(SUM($B$5:$B$12)-SUMPRODUCT($B$5:$B$12,L5:L12)))/(3*SUM($B$5:$B$12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>Unweighted (equal weights, scored criteria only)</t>
+        </is>
+      </c>
+      <c r="C24" s="68">
+        <f>SUM(C5:C12)/(3*COUNT(C5:C12))</f>
+        <v/>
+      </c>
+      <c r="D24" s="68">
+        <f>SUM(D5:D12)/(3*COUNT(D5:D12))</f>
+        <v/>
+      </c>
+      <c r="E24" s="68">
+        <f>SUM(E5:E12)/(3*COUNT(E5:E12))</f>
+        <v/>
+      </c>
+      <c r="F24" s="68">
+        <f>SUM(F5:F12)/(3*COUNT(F5:F12))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="60" t="inlineStr">
+        <is>
+          <t>Rank on headline score (1 = best)</t>
+        </is>
+      </c>
+      <c r="C25" s="63">
+        <f>RANK(C20,$C$20:$F$20)</f>
+        <v/>
+      </c>
+      <c r="D25" s="63">
+        <f>RANK(D20,$C$20:$F$20)</f>
+        <v/>
+      </c>
+      <c r="E25" s="63">
+        <f>RANK(E20,$C$20:$F$20)</f>
+        <v/>
+      </c>
+      <c r="F25" s="63">
+        <f>RANK(F20,$C$20:$F$20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>Security gate (pass/fail, not averaged away)</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>FAIL (Tested)</t>
+        </is>
+      </c>
+      <c r="D26" s="63" t="inlineStr">
+        <is>
+          <t>FAIL as configured (Tested)</t>
+        </is>
+      </c>
+      <c r="E26" s="63" t="inlineStr">
+        <is>
+          <t>Untested (docs: PASS)</t>
+        </is>
+      </c>
+      <c r="F26" s="63" t="inlineStr">
+        <is>
+          <t>Untested (docs: PASS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="64" t="inlineStr">
+        <is>
+          <t>How to read it</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1" s="27">
+      <c r="A29" s="58" t="inlineStr">
+        <is>
+          <t>Headline = weighted points earned / weighted points possible, on the criteria that have a score. It is only comparable between routes if coverage is similar; compare Floor and Ceiling when it is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1" s="27">
+      <c r="A30" s="58" t="inlineStr">
+        <is>
+          <t>Total cost is unscored for every route, so it is excluded from all headline numbers. Security is weighted here, but read the gate row too: a route that fails security can still score well elsewhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1" s="27">
+      <c r="A31" s="58" t="inlineStr">
+        <is>
+          <t>Scores are provisional and from one scorer. Two independent scorers and leadership-set weights are still required before this goes anywhere customer-facing.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A29:G29"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Unguided,Pinned"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>